<commit_message>
Profile Page Failed Test Cases Resolved
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Modules/10_MyHealthBenefits/MyHealthBenefits/01_MyHealthBenefitsTest.xlsx
+++ b/src/test/resources/testdata/Modules/10_MyHealthBenefits/MyHealthBenefits/01_MyHealthBenefitsTest.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\10_MyHealthBenefits\MyHealthBenefits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A2BF7D8-2C08-47C9-ADC3-BEEE99717A16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{978B620C-6810-4DEF-A80C-8A578EE90116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1056" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1056" uniqueCount="262">
   <si>
     <t>INFLUENCER_ACCOUNT</t>
   </si>
@@ -3272,6 +3272,13 @@
 clickon_teleconsulting_arrow
 clickon_mailicon_try
 verify_welcometomail_text</t>
+  </si>
+  <si>
+    <t>navigatebackto_myhealthpage
+clickon_hospicash_arrow
+clickon_videoicon
+clickon_videoicon
+verify_videoprogressbar_isdisplay</t>
   </si>
 </sst>
 </file>
@@ -4513,7 +4520,7 @@
         <v>101</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>102</v>
+        <v>261</v>
       </c>
       <c r="F25" s="21"/>
       <c r="G25" s="21"/>

</xml_diff>